<commit_message>
Updated standard errors to CRN
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -461,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>16326.73152161764</v>
+        <v>28725.35614758425</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>31828.20111957949</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10223.57636852667</v>
+        <v>14928.8320178776</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>14842.66535628654</v>
+        <v>29138.17913844815</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3710.666339071636</v>
+        <v>7284.544784612039</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>47695.33694674358</v>
+        <v>46487.69937914996</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>16218.54965960887</v>
+        <v>11621.98641144057</v>
       </c>
     </row>
     <row r="18">
@@ -839,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>27320.53993629754</v>
+        <v>36844.09611630544</v>
       </c>
     </row>
     <row r="21">
@@ -902,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>27117.48748593112</v>
+        <v>30755.76046864681</v>
       </c>
     </row>
     <row r="24">
@@ -965,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>13821.6562024988</v>
+        <v>10739.47105274393</v>
       </c>
     </row>
     <row r="27">
@@ -1028,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>22805.94811214217</v>
+        <v>23255.36026151579</v>
       </c>
     </row>
     <row r="30">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5701.487028035542</v>
+        <v>5813.840065378947</v>
       </c>
     </row>
     <row r="32">
@@ -1091,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>48287.73173710302</v>
+        <v>43048.73460781306</v>
       </c>
     </row>
     <row r="33">
@@ -1154,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>14869.58287021995</v>
+        <v>10753.51342411154</v>
       </c>
     </row>
     <row r="36">
@@ -1217,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>20052.38353018724</v>
+        <v>26814.71703674526</v>
       </c>
     </row>
     <row r="39">
@@ -1280,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>29882.55738209147</v>
+        <v>10650.39816506652</v>
       </c>
     </row>
     <row r="42">
@@ -1343,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>15713.69505437746</v>
+        <v>6031.558128076127</v>
       </c>
     </row>
     <row r="45">
@@ -1406,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>24194.81956740188</v>
+        <v>16626.27482455417</v>
       </c>
     </row>
     <row r="48">
@@ -1448,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>6048.704891850469</v>
+        <v>4156.568706138542</v>
       </c>
     </row>
     <row r="50">
@@ -1469,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>61265.43247541147</v>
+        <v>34807.53319498364</v>
       </c>
     </row>
     <row r="51">
@@ -1532,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>14243.24615086304</v>
+        <v>13678.42749723228</v>
       </c>
     </row>
     <row r="54">
@@ -1595,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>33800.82186506961</v>
+        <v>18189.81943359092</v>
       </c>
     </row>
     <row r="57">
@@ -1658,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>7962.896620160037</v>
+        <v>14407.72223998532</v>
       </c>
     </row>
     <row r="60">
@@ -1721,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>15701.54734086936</v>
+        <v>17996.18288345583</v>
       </c>
     </row>
     <row r="63">
@@ -1784,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>31852.74516294726</v>
+        <v>18645.34219708079</v>
       </c>
     </row>
     <row r="66">
@@ -1826,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>7963.186290736814</v>
+        <v>4661.335549270197</v>
       </c>
     </row>
     <row r="68">
@@ -1847,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>40671.56787561713</v>
+        <v>51012.92307031886</v>
       </c>
     </row>
     <row r="69">
@@ -1910,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>9748.513031140612</v>
+        <v>7157.194301699537</v>
       </c>
     </row>
     <row r="72">
@@ -1973,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>34647.39259730353</v>
+        <v>20917.12956606113</v>
       </c>
     </row>
     <row r="75">
@@ -2036,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>18049.45495390538</v>
+        <v>25831.91942282399</v>
       </c>
     </row>
     <row r="78">
@@ -2099,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>9999.783827842053</v>
+        <v>8183.774084666365</v>
       </c>
     </row>
     <row r="81">
@@ -2162,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>21019.69111818678</v>
+        <v>22254.18811007404</v>
       </c>
     </row>
     <row r="84">
@@ -2204,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>5254.922779546695</v>
+        <v>5563.547027518509</v>
       </c>
     </row>
     <row r="86">
@@ -2225,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>38015.73184770409</v>
+        <v>40990.41965121793</v>
       </c>
     </row>
     <row r="87">
@@ -2288,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>15781.34188247585</v>
+        <v>11406.14843827521</v>
       </c>
     </row>
     <row r="90">
@@ -2351,7 +2363,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>19068.98408307115</v>
+        <v>20487.20040827952</v>
       </c>
     </row>
     <row r="93">
@@ -2414,7 +2426,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>27704.7501078001</v>
+        <v>38892.08638381703</v>
       </c>
     </row>
     <row r="96">
@@ -2477,7 +2489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>13566.8092362369</v>
+        <v>12449.38540723275</v>
       </c>
     </row>
     <row r="99">
@@ -2540,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>29983.32843445082</v>
+        <v>13653.7344262646</v>
       </c>
     </row>
     <row r="102">
@@ -2582,7 +2594,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>7495.832108612705</v>
+        <v>3413.43360656615</v>
       </c>
     </row>
     <row r="104">
@@ -2603,7 +2615,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>67479.52799443594</v>
+        <v>62338.17368154784</v>
       </c>
     </row>
     <row r="105">
@@ -2666,7 +2678,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>10514.2717195488</v>
+        <v>7921.836312608667</v>
       </c>
     </row>
     <row r="108">
@@ -2729,7 +2741,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>15516.30695145816</v>
+        <v>26566.47696253567</v>
       </c>
     </row>
     <row r="111">
@@ -2792,7 +2804,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>31284.76631483077</v>
+        <v>10302.47407090168</v>
       </c>
     </row>
     <row r="114">
@@ -2855,7 +2867,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>10049.78436967503</v>
+        <v>7519.302316630885</v>
       </c>
     </row>
     <row r="117">
@@ -2918,7 +2930,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>17985.93957257749</v>
+        <v>21181.16741521474</v>
       </c>
     </row>
     <row r="120">
@@ -2960,7 +2972,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>4496.484893144373</v>
+        <v>5295.291853803686</v>
       </c>
     </row>
     <row r="122">
@@ -2981,7 +2993,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>34102.58464904546</v>
+        <v>61076.99869993115</v>
       </c>
     </row>
     <row r="123">
@@ -3044,7 +3056,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>15046.29474045062</v>
+        <v>13142.63105446239</v>
       </c>
     </row>
     <row r="126">
@@ -3107,7 +3119,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>20151.30162671869</v>
+        <v>24132.63788208819</v>
       </c>
     </row>
     <row r="129">
@@ -3170,7 +3182,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>24737.18733772909</v>
+        <v>22741.72228308033</v>
       </c>
     </row>
     <row r="132">
@@ -3233,7 +3245,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>12426.86350290325</v>
+        <v>6955.542536122148</v>
       </c>
     </row>
     <row r="135">
@@ -3296,7 +3308,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>21101.36371948347</v>
+        <v>15680.93474963175</v>
       </c>
     </row>
     <row r="138">
@@ -3338,7 +3350,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>5275.340929870867</v>
+        <v>3920.233687407937</v>
       </c>
     </row>
     <row r="140">
@@ -3359,7 +3371,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>59924.57752579472</v>
+        <v>43090.41843560319</v>
       </c>
     </row>
     <row r="141">
@@ -3422,7 +3434,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>11589.42360539667</v>
+        <v>16464.20834832093</v>
       </c>
     </row>
     <row r="144">

</xml_diff>

<commit_message>
Checked out lognormal distribution, fixed minor issues
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>28725.35614758425</v>
+        <v>24010.30252585355</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>23963.01774121611</v>
+        <v>26157.90753560609</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14928.8320178776</v>
+        <v>10472.0860779841</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29138.17913844815</v>
+        <v>15214.69307332064</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7284.544784612039</v>
+        <v>3803.673268330159</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46487.69937914996</v>
+        <v>4820.236059577976</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11621.98641144057</v>
+        <v>15117.12986779355</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>36844.09611630544</v>
+        <v>24647.04253768335</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>30755.76046864681</v>
+        <v>33634.23279277765</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10739.47105274393</v>
+        <v>11765.21460077968</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>23255.36026151579</v>
+        <v>24964.1524655337</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5813.840065378947</v>
+        <v>6241.038116383425</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>43048.73460781306</v>
+        <v>42736.33864021432</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10753.51342411154</v>
+        <v>11802.5160791596</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>26814.71703674526</v>
+        <v>26935.25828712281</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>10650.39816506652</v>
+        <v>37146.45144822418</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>6031.558128076127</v>
+        <v>14913.45688528014</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>16626.27482455417</v>
+        <v>9956.85769416782</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4156.568706138542</v>
+        <v>2489.214423541955</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>34807.53319498364</v>
+        <v>56002.35466296331</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>13678.42749723228</v>
+        <v>6458.574109742418</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>18189.81943359092</v>
+        <v>15385.81175494</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>14407.72223998532</v>
+        <v>46843.81414575673</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>17996.18288345583</v>
+        <v>7295.505209794742</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>18645.34219708079</v>
+        <v>20863.03838132927</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>4661.335549270197</v>
+        <v>5215.759595332318</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>51012.92307031886</v>
+        <v>41736.64931756931</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>7157.194301699537</v>
+        <v>11759.08810485141</v>
       </c>
     </row>
     <row r="72">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>20917.12956606113</v>
+        <v>13804.93788034449</v>
       </c>
     </row>
     <row r="75">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>25831.91942282399</v>
+        <v>41245.57086843469</v>
       </c>
     </row>
     <row r="78">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>8183.774084666365</v>
+        <v>14861.79625743754</v>
       </c>
     </row>
     <row r="81">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>22254.18811007404</v>
+        <v>12106.04534809321</v>
       </c>
     </row>
     <row r="84">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>5563.547027518509</v>
+        <v>3026.511337023303</v>
       </c>
     </row>
     <row r="86">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>40990.41965121793</v>
+        <v>43595.35674313323</v>
       </c>
     </row>
     <row r="87">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>11406.14843827521</v>
+        <v>17878.44008749364</v>
       </c>
     </row>
     <row r="90">
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>20487.20040827952</v>
+        <v>19372.63050329489</v>
       </c>
     </row>
     <row r="93">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>38892.08638381703</v>
+        <v>33948.66718518956</v>
       </c>
     </row>
     <row r="96">
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>12449.38540723275</v>
+        <v>12383.39681508774</v>
       </c>
     </row>
     <row r="99">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>13653.7344262646</v>
+        <v>24426.03804597851</v>
       </c>
     </row>
     <row r="102">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>3413.43360656615</v>
+        <v>6106.509511494627</v>
       </c>
     </row>
     <row r="104">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>62338.17368154784</v>
+        <v>44573.28192042394</v>
       </c>
     </row>
     <row r="105">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>7921.836312608667</v>
+        <v>11674.48280505801</v>
       </c>
     </row>
     <row r="108">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>26566.47696253567</v>
+        <v>26240.43988901527</v>
       </c>
     </row>
     <row r="111">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>10302.47407090168</v>
+        <v>36382.46473074835</v>
       </c>
     </row>
     <row r="114">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>7519.302316630885</v>
+        <v>7065.448594888454</v>
       </c>
     </row>
     <row r="117">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>21181.16741521474</v>
+        <v>25179.95561460332</v>
       </c>
     </row>
     <row r="120">
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>5295.291853803686</v>
+        <v>6294.98890365083</v>
       </c>
     </row>
     <row r="122">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>61076.99869993115</v>
+        <v>53622.96612418298</v>
       </c>
     </row>
     <row r="123">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>13142.63105446239</v>
+        <v>12865.60500611564</v>
       </c>
     </row>
     <row r="126">
@@ -3119,7 +3119,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>24132.63788208819</v>
+        <v>30056.00031156575</v>
       </c>
     </row>
     <row r="129">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>22741.72228308033</v>
+        <v>13010.40747639669</v>
       </c>
     </row>
     <row r="132">
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>6955.542536122148</v>
+        <v>9137.912668342355</v>
       </c>
     </row>
     <row r="135">
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>15680.93474963175</v>
+        <v>28513.14788855238</v>
       </c>
     </row>
     <row r="138">
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>3920.233687407937</v>
+        <v>7128.286972138094</v>
       </c>
     </row>
     <row r="140">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>43090.41843560319</v>
+        <v>61395.3337578938</v>
       </c>
     </row>
     <row r="141">
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>16464.20834832093</v>
+        <v>15851.75363024716</v>
       </c>
     </row>
     <row r="144">

</xml_diff>

<commit_message>
Made an experiment utils
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>24010.30252585355</v>
+        <v>26679.84192246049</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26157.90753560609</v>
+        <v>16896.80823734788</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10472.0860779841</v>
+        <v>11503.18948121408</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>15214.69307332064</v>
+        <v>23363.36400882185</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3803.673268330159</v>
+        <v>5840.841002205463</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4820.236059577976</v>
+        <v>34356.45818706114</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>15117.12986779355</v>
+        <v>11688.73528438797</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>24647.04253768335</v>
+        <v>20437.82972754275</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>33634.23279277765</v>
+        <v>18484.28952263853</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>11765.21460077968</v>
+        <v>15596.15974053148</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>24964.1524655337</v>
+        <v>25674.23883259048</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>6241.038116383425</v>
+        <v>6418.55970814762</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>42736.33864021432</v>
+        <v>50070.25844885917</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>11802.5160791596</v>
+        <v>15397.01245939138</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>26935.25828712281</v>
+        <v>19935.13198309845</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>37146.45144822418</v>
+        <v>24917.32850328527</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>14913.45688528014</v>
+        <v>4083.238851101151</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>9956.85769416782</v>
+        <v>16905.45414662882</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2489.214423541955</v>
+        <v>4226.363536657206</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>56002.35466296331</v>
+        <v>73649.20158374368</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>6458.574109742418</v>
+        <v>12236.57336912522</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>15385.81175494</v>
+        <v>27719.43470477354</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>46843.81414575673</v>
+        <v>18504.87358996176</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>7295.505209794742</v>
+        <v>20091.73003969418</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>20863.03838132927</v>
+        <v>27754.63092221083</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>5215.759595332318</v>
+        <v>6938.657730552707</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>41736.64931756931</v>
+        <v>29510.31593098802</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>11759.08810485141</v>
+        <v>12905.73286185439</v>
       </c>
     </row>
     <row r="72">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>13804.93788034449</v>
+        <v>23737.27271101013</v>
       </c>
     </row>
     <row r="75">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>41245.57086843469</v>
+        <v>22982.20685072818</v>
       </c>
     </row>
     <row r="78">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>14861.79625743754</v>
+        <v>4232.512627570363</v>
       </c>
     </row>
     <row r="81">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>12106.04534809321</v>
+        <v>16049.77377966454</v>
       </c>
     </row>
     <row r="84">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>3026.511337023303</v>
+        <v>4012.443444916134</v>
       </c>
     </row>
     <row r="86">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>43595.35674313323</v>
+        <v>46303.29557605527</v>
       </c>
     </row>
     <row r="87">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>17878.44008749364</v>
+        <v>16471.8663050594</v>
       </c>
     </row>
     <row r="90">
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>19372.63050329489</v>
+        <v>15863.1338260768</v>
       </c>
     </row>
     <row r="93">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>33948.66718518956</v>
+        <v>26883.77423678695</v>
       </c>
     </row>
     <row r="96">
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>12383.39681508774</v>
+        <v>11867.85995460826</v>
       </c>
     </row>
     <row r="99">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>24426.03804597851</v>
+        <v>5271.455580312555</v>
       </c>
     </row>
     <row r="102">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>6106.509511494627</v>
+        <v>1317.863895078139</v>
       </c>
     </row>
     <row r="104">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>44573.28192042394</v>
+        <v>54745.22182523392</v>
       </c>
     </row>
     <row r="105">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>11674.48280505801</v>
+        <v>15861.16033408308</v>
       </c>
     </row>
     <row r="108">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>26240.43988901527</v>
+        <v>22333.01848797451</v>
       </c>
     </row>
     <row r="111">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>36382.46473074835</v>
+        <v>23411.48885087506</v>
       </c>
     </row>
     <row r="114">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>7065.448594888454</v>
+        <v>11843.33296129047</v>
       </c>
     </row>
     <row r="117">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>25179.95561460332</v>
+        <v>16793.52848941435</v>
       </c>
     </row>
     <row r="120">
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>6294.98890365083</v>
+        <v>4198.382122353587</v>
       </c>
     </row>
     <row r="122">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>53622.96612418298</v>
+        <v>42853.475019366</v>
       </c>
     </row>
     <row r="123">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>12865.60500611564</v>
+        <v>15905.54243878526</v>
       </c>
     </row>
     <row r="126">
@@ -3119,7 +3119,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>30056.00031156575</v>
+        <v>26455.91116069835</v>
       </c>
     </row>
     <row r="129">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>13010.40747639669</v>
+        <v>16779.50458944508</v>
       </c>
     </row>
     <row r="132">
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>9137.912668342355</v>
+        <v>13573.61048990052</v>
       </c>
     </row>
     <row r="135">
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>28513.14788855238</v>
+        <v>25105.78719334343</v>
       </c>
     </row>
     <row r="138">
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>7128.286972138094</v>
+        <v>6276.446798335858</v>
       </c>
     </row>
     <row r="140">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>61395.3337578938</v>
+        <v>52528.63775255777</v>
       </c>
     </row>
     <row r="141">
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>15851.75363024716</v>
+        <v>13950.7680751837</v>
       </c>
     </row>
     <row r="144">

</xml_diff>

<commit_message>
Added alternative price and demand sampling possibility
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>26679.84192246049</v>
+        <v>18340.15324983363</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>16896.80823734788</v>
+        <v>20465.83582367539</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>11503.18948121408</v>
+        <v>10605.75129696297</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>23363.36400882185</v>
+        <v>34562.11979913599</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5840.841002205463</v>
+        <v>8640.529949783997</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>34356.45818706114</v>
+        <v>42097.90922628069</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11688.73528438797</v>
+        <v>13685.0446900253</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>20437.82972754275</v>
+        <v>18591.65514489271</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>18484.28952263853</v>
+        <v>23087.54948832049</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>15596.15974053148</v>
+        <v>9985.055606659849</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>25674.23883259048</v>
+        <v>14753.59746168853</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>6418.55970814762</v>
+        <v>3688.399365422134</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>50070.25844885917</v>
+        <v>45682.75770723016</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>15397.01245939138</v>
+        <v>10649.09843423136</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>19935.13198309845</v>
+        <v>31042.20486162991</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>24917.32850328527</v>
+        <v>28187.85393779481</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>4083.238851101151</v>
+        <v>15308.52740868841</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>16905.45414662882</v>
+        <v>24283.47324629944</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4226.363536657206</v>
+        <v>6070.868311574859</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>73649.20158374368</v>
+        <v>50596.49847488942</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>12236.57336912522</v>
+        <v>19485.50333601054</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>27719.43470477354</v>
+        <v>36110.04212563561</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>18504.87358996176</v>
+        <v>37511.08287569358</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>20091.73003969418</v>
+        <v>16128.69865070354</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>27754.63092221083</v>
+        <v>37260.62623705292</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>6938.657730552707</v>
+        <v>9315.156559263231</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>29510.31593098802</v>
+        <v>40378.45907060537</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>12905.73286185439</v>
+        <v>15708.89078961611</v>
       </c>
     </row>
     <row r="72">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>23737.27271101013</v>
+        <v>32221.22850694642</v>
       </c>
     </row>
     <row r="75">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>22982.20685072818</v>
+        <v>17502.58745192984</v>
       </c>
     </row>
     <row r="78">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>4232.512627570363</v>
+        <v>9475.775439236009</v>
       </c>
     </row>
     <row r="81">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>16049.77377966454</v>
+        <v>22277.3676796589</v>
       </c>
     </row>
     <row r="84">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>4012.443444916134</v>
+        <v>5569.341919914726</v>
       </c>
     </row>
     <row r="86">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>46303.29557605527</v>
+        <v>63457.0116714217</v>
       </c>
     </row>
     <row r="87">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>16471.8663050594</v>
+        <v>13105.55440986888</v>
       </c>
     </row>
     <row r="90">
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>15863.1338260768</v>
+        <v>29335.35212220977</v>
       </c>
     </row>
     <row r="93">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>26883.77423678695</v>
+        <v>24588.76104715524</v>
       </c>
     </row>
     <row r="96">
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>11867.85995460826</v>
+        <v>11401.42668442093</v>
       </c>
     </row>
     <row r="99">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>5271.455580312555</v>
+        <v>15622.08634937179</v>
       </c>
     </row>
     <row r="102">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>1317.863895078139</v>
+        <v>3905.521587342947</v>
       </c>
     </row>
     <row r="104">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>54745.22182523392</v>
+        <v>32705.16869871289</v>
       </c>
     </row>
     <row r="105">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>15861.16033408308</v>
+        <v>13889.63413110446</v>
       </c>
     </row>
     <row r="108">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>22333.01848797451</v>
+        <v>17787.49467201403</v>
       </c>
     </row>
     <row r="111">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>23411.48885087506</v>
+        <v>18057.07830592771</v>
       </c>
     </row>
     <row r="114">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>11843.33296129047</v>
+        <v>11211.73414764568</v>
       </c>
     </row>
     <row r="117">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>16793.52848941435</v>
+        <v>25498.1611617471</v>
       </c>
     </row>
     <row r="120">
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>4198.382122353587</v>
+        <v>6374.540290436775</v>
       </c>
     </row>
     <row r="122">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>42853.475019366</v>
+        <v>46308.42159578404</v>
       </c>
     </row>
     <row r="123">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>15905.54243878526</v>
+        <v>12621.7245686445</v>
       </c>
     </row>
     <row r="126">
@@ -3119,7 +3119,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>26455.91116069835</v>
+        <v>14821.81256065552</v>
       </c>
     </row>
     <row r="129">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>16779.50458944508</v>
+        <v>19974.30302399116</v>
       </c>
     </row>
     <row r="132">
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>13573.61048990052</v>
+        <v>11816.56064727389</v>
       </c>
     </row>
     <row r="135">
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>25105.78719334343</v>
+        <v>22638.71557864445</v>
       </c>
     </row>
     <row r="138">
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>6276.446798335858</v>
+        <v>5659.678894661112</v>
       </c>
     </row>
     <row r="140">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>52528.63775255777</v>
+        <v>52106.52760579947</v>
       </c>
     </row>
     <row r="141">
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>13950.7680751837</v>
+        <v>11215.99992731266</v>
       </c>
     </row>
     <row r="144">

</xml_diff>

<commit_message>
Prepared subsidy experiment new lognormal demand
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios188.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>18340.15324983363</v>
+        <v>27704.71379621089</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>20465.83582367539</v>
+        <v>22993.18933169442</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10605.75129696297</v>
+        <v>14480.10283854169</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>34562.11979913599</v>
+        <v>29956.44962014933</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>8640.529949783997</v>
+        <v>7489.112405037332</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>42097.90922628069</v>
+        <v>44709.94695541648</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>13685.0446900253</v>
+        <v>11177.54061008852</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>18591.65514489271</v>
+        <v>38068.27620371435</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>23087.54948832049</v>
+        <v>29996.34097896187</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>9985.055606659849</v>
+        <v>10431.40239120233</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>14753.59746168853</v>
+        <v>22464.07929196216</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3688.399365422134</v>
+        <v>5616.01982299054</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>45682.75770723016</v>
+        <v>41799.86390539659</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10649.09843423136</v>
+        <v>10442.87568333659</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>31042.20486162991</v>
+        <v>25708.39296093324</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>28187.85393779481</v>
+        <v>13655.24507760699</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>15308.52740868841</v>
+        <v>7215.794205582797</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>24283.47324629944</v>
+        <v>16241.63626878765</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>6070.868311574859</v>
+        <v>4060.409067196913</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>50596.49847488942</v>
+        <v>35573.71667537648</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>19485.50333601054</v>
+        <v>13129.87755012481</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>36110.04212563561</v>
+        <v>18342.61580025829</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>37511.08287569358</v>
+        <v>15818.66491615211</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>16128.69865070354</v>
+        <v>18410.0406738813</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>37260.62623705292</v>
+        <v>17928.01277455997</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>9315.156559263231</v>
+        <v>4482.003193639992</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>40378.45907060537</v>
+        <v>48850.1653181706</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>15708.89078961611</v>
+        <v>7880.490738312205</v>
       </c>
     </row>
     <row r="72">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>32221.22850694642</v>
+        <v>20409.03668868938</v>
       </c>
     </row>
     <row r="75">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>17502.58745192984</v>
+        <v>24738.22094330983</v>
       </c>
     </row>
     <row r="78">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>9475.775439236009</v>
+        <v>8539.937464649229</v>
       </c>
     </row>
     <row r="81">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>22277.3676796589</v>
+        <v>21390.21294006276</v>
       </c>
     </row>
     <row r="84">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>5569.341919914726</v>
+        <v>5347.553235015691</v>
       </c>
     </row>
     <row r="86">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>63457.0116714217</v>
+        <v>40149.51801559223</v>
       </c>
     </row>
     <row r="87">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>13105.55440986888</v>
+        <v>10990.26705991647</v>
       </c>
     </row>
     <row r="90">
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>29335.35212220977</v>
+        <v>20068.46656369309</v>
       </c>
     </row>
     <row r="93">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>24588.76104715524</v>
+        <v>41245.51843967277</v>
       </c>
     </row>
     <row r="96">
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>11401.42668442093</v>
+        <v>11925.48307962132</v>
       </c>
     </row>
     <row r="99">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>15622.08634937179</v>
+        <v>14043.24369099732</v>
       </c>
     </row>
     <row r="102">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>3905.521587342947</v>
+        <v>3510.810922749331</v>
       </c>
     </row>
     <row r="104">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>32705.16869871289</v>
+        <v>60971.14708213728</v>
       </c>
     </row>
     <row r="105">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>13889.63413110446</v>
+        <v>8366.607379658408</v>
       </c>
     </row>
     <row r="108">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>17787.49467201403</v>
+        <v>25459.80802649001</v>
       </c>
     </row>
     <row r="111">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>18057.07830592771</v>
+        <v>13470.54529866928</v>
       </c>
     </row>
     <row r="114">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>11211.73414764568</v>
+        <v>8107.073855171791</v>
       </c>
     </row>
     <row r="117">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>25498.1611617471</v>
+        <v>20296.20828247051</v>
       </c>
     </row>
     <row r="120">
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>6374.540290436775</v>
+        <v>5074.052070617628</v>
       </c>
     </row>
     <row r="122">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>46308.42159578404</v>
+        <v>59484.67322810461</v>
       </c>
     </row>
     <row r="123">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>12621.7245686445</v>
+        <v>12590.55253361479</v>
       </c>
     </row>
     <row r="126">
@@ -3119,7 +3119,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>14821.81256065552</v>
+        <v>23146.35283311673</v>
       </c>
     </row>
     <row r="129">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>19974.30302399116</v>
+        <v>21919.89915967395</v>
       </c>
     </row>
     <row r="132">
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>11816.56064727389</v>
+        <v>7757.067164419483</v>
       </c>
     </row>
     <row r="135">
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>22638.71557864445</v>
+        <v>15507.52960044835</v>
       </c>
     </row>
     <row r="138">
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>5659.678894661112</v>
+        <v>3876.882400112087</v>
       </c>
     </row>
     <row r="140">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>52106.52760579947</v>
+        <v>41833.97736759408</v>
       </c>
     </row>
     <row r="141">
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>11215.99992731266</v>
+        <v>16329.42994277851</v>
       </c>
     </row>
     <row r="144">

</xml_diff>